<commit_message>
docs(roadmap): update NOVA R01 R02 R05 status
</commit_message>
<xml_diff>
--- a/Docs/00_GOVERNANCE/PROJECT_TRACKING/NOVA_ROADMAP_GANTT_2026-09-29.xlsx
+++ b/Docs/00_GOVERNANCE/PROJECT_TRACKING/NOVA_ROADMAP_GANTT_2026-09-29.xlsx
@@ -937,7 +937,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Figer la baseline as-built et le registre des gaps actuels</t>
+          <t>Figer l'état réel actuel de NOVA et le registre des écarts.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -953,12 +953,12 @@
       <c r="F5" s="4"/>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROGRAM-003 réconcilié ; WCF-008 certifié ; audit as-built en cours</t>
+          <t>Baseline figée sur feature/nova-runtime-foundation au commit 3ebf5ba689e4df2f2309e8dd31f34093d243237b. Worktree propre. Architecture vérifiée : UI -&gt; BFF -&gt; NOVA Core HTTP -&gt; Mission/Runtime. Registre des écarts consolidé.</t>
         </is>
       </c>
       <c r="I5" s="23">
@@ -970,8 +970,10 @@
       <c r="K5" s="24">
         <f>I5+J5-1</f>
       </c>
-      <c r="L5" s="7">
-        <f>IF(G5="Terminé",1,IF(G5="En cours",0.5,0))</f>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
       </c>
       <c r="M5" s="8">
         <f>IF(OR(G5="Terminé",K5=""),0,MAX(0,TODAY()-K5))</f>
@@ -999,7 +1001,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assembler ProgramProductionEntrypoint dans le BFF réellement lancé</t>
+          <t>Raccorder le BFF à l'autorité Mission/Runtime de NOVA Core via HTTP, sans créer de seconde autorité d'exécution.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1019,12 +1021,12 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Composants présents séparément ; start:bff n'injecte pas RuntimeGateway</t>
+          <t>R01/R02 : NOVA Core expose déjà POST /api/v1/missions et POST /api/v1/missions/{projectId}/{missionId}/execute. BFF_RUNTIME_ORIGIN pointe vers NOVA Core :4100. Les gateways HTTP de lecture existent. Le runtimeGateway historique n'est pas injecté et son contrat ProgramProductionEntrypoint ne correspond pas directement au contrat Mission/Runtime actuel. Développement minimal attendu : passerelle BFF dédiée Mission/Runtime. Ne pas modifier NOVA Core ni créer un second moteur.</t>
         </is>
       </c>
       <c r="I6" s="23">
@@ -1036,8 +1038,10 @@
       <c r="K6" s="24">
         <f>I6+J6-1</f>
       </c>
-      <c r="L6" s="7">
-        <f>IF(G6="Terminé",1,IF(G6="En cours",0.5,0))</f>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
       </c>
       <c r="M6" s="8">
         <f>IF(OR(G6="Terminé",K6=""),0,MAX(0,TODAY()-K6))</f>
@@ -1197,7 +1201,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brancher Confirm → exécution Mission/Runtime existante</t>
+          <t>Connecter Confirm à la passerelle BFF Mission/Runtime existante afin de créer/lancer la Mission puis ouvrir le Work réel.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1217,12 +1221,12 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t>À faire</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ne pas créer de nouveau Create Work ; réutiliser Mission/Runtime</t>
+          <t>ConfirmPage utilise actuellement navigate('work') uniquement. R05 dépend de R02. L'autorité de création reste Mission/Runtime ; aucun moteur Create Work indépendant ne doit être créé.</t>
         </is>
       </c>
       <c r="I9" s="23">
@@ -1234,8 +1238,10 @@
       <c r="K9" s="24">
         <f>I9+J9-1</f>
       </c>
-      <c r="L9" s="7">
-        <f>IF(G9="Terminé",1,IF(G9="En cours",0.5,0))</f>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
       </c>
       <c r="M9" s="8">
         <f>IF(OR(G9="Terminé",K9=""),0,MAX(0,TODAY()-K9))</f>

</xml_diff>

<commit_message>
feat(tracking): sync final authority decisions
</commit_message>
<xml_diff>
--- a/Docs/00_GOVERNANCE/PROJECT_TRACKING/NOVA_ROADMAP_GANTT_2026-09-29.xlsx
+++ b/Docs/00_GOVERNANCE/PROJECT_TRACKING/NOVA_ROADMAP_GANTT_2026-09-29.xlsx
@@ -13489,7 +13489,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
@@ -13526,7 +13526,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
@@ -13563,7 +13563,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
@@ -13600,14 +13600,14 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NOVA-SUPER-WAVE-RT12-PROVENANCE-CLOSURE-001</t>
+          <t>NOVA-R02-BFF-MISSION-RUNTIME-HTTP-BRIDGE-001</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -13617,34 +13617,34 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PENDING_REVIEW</t>
+          <t>ACCEPTED</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>ACCEPTED</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CC9AD198EDB08AC8AF64CF2658789F4C7553353485A6E86D6BAB0DEBBC7D16F5</t>
+          <t>A4ED0525EBA487AD8EA400DA41A9023216E9EAB5DCDBF8EDF9C2ACC64A2E8825</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-SUPER-WAVE-RT12-PROVENANCE-CLOSURE-001\bootstrap-20260917T160907003\official-report.json</t>
+          <t>.nova-data\execution\reports\NOVA-AS-BUILT-COMPLETION\NOVA-R02-BFF-MISSION-RUNTIME-HTTP-BRIDGE-001\bootstrap-20260929T175046117\official-report.json</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NOVA-WORK-CERTIFICATION-FINAL-CLOSURE-001</t>
+          <t>NOVA-SUPER-WAVE-RT12-PROVENANCE-CLOSURE-001</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -13664,24 +13664,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>B08AC39DD5A194D049E743140B5D952C91A2262D0C1C0392B79E78A39778F888</t>
+          <t>CC9AD198EDB08AC8AF64CF2658789F4C7553353485A6E86D6BAB0DEBBC7D16F5</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-CERTIFICATION-FINAL-CLOSURE-001\bootstrap-20260919T162258742\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-SUPER-WAVE-RT12-PROVENANCE-CLOSURE-001\bootstrap-20260917T160907003\official-report.json</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NOVA-WORK-WCF008-C19-RED-TEAM-REVALIDATION-001</t>
+          <t>NOVA-WORK-CERTIFICATION-FINAL-CLOSURE-001</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -13701,24 +13701,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>F523C276F31EBDF077F882AF67E9D65B650ED26B3497667EB547A8B560D6A8EA</t>
+          <t>B08AC39DD5A194D049E743140B5D952C91A2262D0C1C0392B79E78A39778F888</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C19-RED-TEAM-REVALIDATION-001\bootstrap-20260928T141436900\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-CERTIFICATION-FINAL-CLOSURE-001\bootstrap-20260919T162258742\official-report.json</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>NOVA-WORK-WCF008-C20-OFFICIAL-REPORT-SEAL-AUDIT-001</t>
+          <t>NOVA-WORK-WCF008-C19-RED-TEAM-REVALIDATION-001</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -13738,24 +13738,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4C7F0ED1FD77F57332E1591404779737266EB71921180CC56BD04FF82CBB961E</t>
+          <t>F523C276F31EBDF077F882AF67E9D65B650ED26B3497667EB547A8B560D6A8EA</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C20-OFFICIAL-REPORT-SEAL-AUDIT-001\bootstrap-20260928T160351555\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C19-RED-TEAM-REVALIDATION-001\bootstrap-20260928T141436900\official-report.json</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NOVA-WORK-WCF008-C21-FINAL-CLOSURE-READINESS-001</t>
+          <t>NOVA-WORK-WCF008-C20-OFFICIAL-REPORT-SEAL-AUDIT-001</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -13770,29 +13770,29 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>22C04477C91C196702DDD99184A975A46DACDE8EBE20F6C679B1477A33861EA9</t>
+          <t>4C7F0ED1FD77F57332E1591404779737266EB71921180CC56BD04FF82CBB961E</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C21-FINAL-CLOSURE-READINESS-001\bootstrap-20260928T233841880\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C20-OFFICIAL-REPORT-SEAL-AUDIT-001\bootstrap-20260928T160351555\official-report.json</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NOVA-WORK-WCF008-FINAL-PRE-C21-VALIDATION-001</t>
+          <t>NOVA-WORK-WCF008-C21-FINAL-CLOSURE-READINESS-001</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -13807,29 +13807,29 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>CERTIFIED</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>E23ED2A88B1C3B2650B66694C6AD9F498A1086E05DF287727C1C1EF3F74C0186</t>
+          <t>22C04477C91C196702DDD99184A975A46DACDE8EBE20F6C679B1477A33861EA9</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\NOVA\NOVA-WORK-WCF008-FINAL-PRE-C21-VALIDATION-001\bootstrap-20260928T102331010\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C21-FINAL-CLOSURE-READINESS-001\bootstrap-20260928T233841880\official-report.json</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001A-IMPLEMENTATION-CONTRACT</t>
+          <t>NOVA-WORK-WCF008-FINAL-PRE-C21-VALIDATION-001</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -13849,24 +13849,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BF26635526F1076CEAA9025E859DF3AEDFC5484E116FF1DC01B041508921B96F</t>
+          <t>E23ED2A88B1C3B2650B66694C6AD9F498A1086E05DF287727C1C1EF3F74C0186</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001A-IMPLEMENTATION-CONTRACT\bootstrap-20260908T102551406\official-report.json</t>
+          <t>.nova-data\execution\reports\NOVA\NOVA-WORK-WCF008-FINAL-PRE-C21-VALIDATION-001\bootstrap-20260928T102331010\official-report.json</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001B-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001A-IMPLEMENTATION-CONTRACT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -13881,29 +13881,29 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1D55CAFE5144E3B7EC41C6F41E7E7233A692F14EA0C15B23E5ABC7DC6D0F5CD5</t>
+          <t>BF26635526F1076CEAA9025E859DF3AEDFC5484E116FF1DC01B041508921B96F</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001B-IMPLEMENTATION-001\bootstrap-20260908T164222685\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001A-IMPLEMENTATION-CONTRACT\bootstrap-20260908T102551406\official-report.json</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001C-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -13923,24 +13923,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>351FC47C1FD4CA8E66AF7DD143A084DD1C14EB89384F00B37FFFDFD63949F352</t>
+          <t>1D55CAFE5144E3B7EC41C6F41E7E7233A692F14EA0C15B23E5ABC7DC6D0F5CD5</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001C-IMPLEMENTATION-001\bootstrap-20260910T105924679\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001B-IMPLEMENTATION-001\bootstrap-20260908T164222685\official-report.json</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001D-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001C-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -13960,24 +13960,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>27DAF65D046D7132AB457F8768ABCB22812E4ABA85BB9248B3BC79AD18C7FE29</t>
+          <t>351FC47C1FD4CA8E66AF7DD143A084DD1C14EB89384F00B37FFFDFD63949F352</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001D-IMPLEMENTATION-001\bootstrap-20260910T132750068\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001C-IMPLEMENTATION-001\bootstrap-20260910T105924679\official-report.json</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001E-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001D-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -13997,24 +13997,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>8B1BC8B78FAD692F07C02EEBFE3702E2BBB75CAD46E49CAD91860263389789EA</t>
+          <t>27DAF65D046D7132AB457F8768ABCB22812E4ABA85BB9248B3BC79AD18C7FE29</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001E-IMPLEMENTATION-001\bootstrap-20260910T163042722\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001D-IMPLEMENTATION-001\bootstrap-20260910T132750068\official-report.json</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001F-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001E-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -14034,24 +14034,24 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>D7B20722E39CF6C3187472CB67E23388D00419EB08E7DDD6F7C167734F515FC9</t>
+          <t>8B1BC8B78FAD692F07C02EEBFE3702E2BBB75CAD46E49CAD91860263389789EA</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001F-IMPLEMENTATION-001\bootstrap-20260910T234329189\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001E-IMPLEMENTATION-001\bootstrap-20260910T163042722\official-report.json</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001G-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001F-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -14071,24 +14071,24 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5525B5851E6F2C1A8D02ADB45FAE10A6D85435164EEE5C44552E06C055395D31</t>
+          <t>D7B20722E39CF6C3187472CB67E23388D00419EB08E7DDD6F7C167734F515FC9</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001G-IMPLEMENTATION-001\bootstrap-20260913T195219085\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001F-IMPLEMENTATION-001\bootstrap-20260910T234329189\official-report.json</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>P3-BUSINESS-CERTIFICATION-001B-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001G-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -14108,24 +14108,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>32DD5DC8698BEA0E159E4C7F5E22852791A59CF119BA967C5B912823DAFF2343</t>
+          <t>5525B5851E6F2C1A8D02ADB45FAE10A6D85435164EEE5C44552E06C055395D31</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-BUSINESS-CERTIFICATION-001B-IMPLEMENTATION-001\bootstrap-20260917T150647587\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001G-IMPLEMENTATION-001\bootstrap-20260913T195219085\official-report.json</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>P3-CONFIDENCE-001B-IMPLEMENTATION-001</t>
+          <t>P3-BUSINESS-CERTIFICATION-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -14145,24 +14145,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>DB4A6A3AFAEC0C7C91C3A4E4B523603D6752A8734826F01076C249B1337706FE</t>
+          <t>32DD5DC8698BEA0E159E4C7F5E22852791A59CF119BA967C5B912823DAFF2343</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-CONFIDENCE-001B-IMPLEMENTATION-001\bootstrap-20260918T125752601\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-BUSINESS-CERTIFICATION-001B-IMPLEMENTATION-001\bootstrap-20260917T150647587\official-report.json</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>P3-EVIDENCE-001B-IMPLEMENTATION-001</t>
+          <t>P3-CONFIDENCE-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -14182,24 +14182,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>37A4453AA09E7157A2D12D5DF1FE0526163A252E4745435A1A18E80F9DEB29E0</t>
+          <t>DB4A6A3AFAEC0C7C91C3A4E4B523603D6752A8734826F01076C249B1337706FE</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-EVIDENCE-001B-IMPLEMENTATION-001\bootstrap-20260915T130433792\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-CONFIDENCE-001B-IMPLEMENTATION-001\bootstrap-20260918T125752601\official-report.json</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>P3-INTELLIGENCE-001B-IMPLEMENTATION-001</t>
+          <t>P3-EVIDENCE-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -14219,24 +14219,24 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>576375263E1D11F4D9BC49929BA0A701C645C387430AE1EAB711A1D9C71713C5</t>
+          <t>37A4453AA09E7157A2D12D5DF1FE0526163A252E4745435A1A18E80F9DEB29E0</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-INTELLIGENCE-001B-IMPLEMENTATION-001\bootstrap-20260917T205856790\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-EVIDENCE-001B-IMPLEMENTATION-001\bootstrap-20260915T130433792\official-report.json</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001C-FINAL-EVIDENCE-002</t>
+          <t>P3-INTELLIGENCE-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -14256,24 +14256,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>14D7FCEF0C6EE5ABAE5B3052A19508CDCD01B420EDA2E21F07120E79006B3167</t>
+          <t>576375263E1D11F4D9BC49929BA0A701C645C387430AE1EAB711A1D9C71713C5</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001C-FINAL-EVIDENCE-002\bootstrap-20260905T180227989\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-INTELLIGENCE-001B-IMPLEMENTATION-001\bootstrap-20260917T205856790\official-report.json</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001D-IMPLEMENTATION-001</t>
+          <t>P3-PLANNING-001C-FINAL-EVIDENCE-002</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -14293,24 +14293,24 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0442A6023581D62C7B7FA926BE258027452B03149D42C3B2AE4BA7ABBA64E243</t>
+          <t>14D7FCEF0C6EE5ABAE5B3052A19508CDCD01B420EDA2E21F07120E79006B3167</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001D-IMPLEMENTATION-001\bootstrap-20260905T190028578\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001C-FINAL-EVIDENCE-002\bootstrap-20260905T180227989\official-report.json</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001E-IMPLEMENTATION-001</t>
+          <t>P3-PLANNING-001D-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -14330,24 +14330,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>67BCE4021666AA8C5B5A2DED6BC88FD54DEF839EDA9F4ED8E28EBE76AD40D119</t>
+          <t>0442A6023581D62C7B7FA926BE258027452B03149D42C3B2AE4BA7ABBA64E243</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001E-IMPLEMENTATION-001\bootstrap-20260906T193230204\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001D-IMPLEMENTATION-001\bootstrap-20260905T190028578\official-report.json</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001F-IMPLEMENTATION-001</t>
+          <t>P3-PLANNING-001E-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -14367,24 +14367,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2D9CAF4114AE784DD95CD5471132144ADC8FADF6CACC56A94833DDF5192DE82C</t>
+          <t>67BCE4021666AA8C5B5A2DED6BC88FD54DEF839EDA9F4ED8E28EBE76AD40D119</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001F-IMPLEMENTATION-001\bootstrap-20260906T213644505\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001E-IMPLEMENTATION-001\bootstrap-20260906T193230204\official-report.json</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001G-IMPLEMENTATION-001</t>
+          <t>P3-PLANNING-001F-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -14404,24 +14404,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>B1068CA311366D7BB4DD626606C435E73F720494212448686615A821311D6DBF</t>
+          <t>2D9CAF4114AE784DD95CD5471132144ADC8FADF6CACC56A94833DDF5192DE82C</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001G-IMPLEMENTATION-001\bootstrap-20260907T174646937\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001F-IMPLEMENTATION-001\bootstrap-20260906T213644505\official-report.json</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>P3-SYNTHESIS-001B-IMPLEMENTATION-001</t>
+          <t>P3-PLANNING-001G-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -14441,24 +14441,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>A456BAD939D4206681D2203DA4D0CE674D5510A7989E9EF8730820E08F76F30E</t>
+          <t>B1068CA311366D7BB4DD626606C435E73F720494212448686615A821311D6DBF</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-SYNTHESIS-001B-IMPLEMENTATION-001\bootstrap-20260917T230506107\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001G-IMPLEMENTATION-001\bootstrap-20260907T174646937\official-report.json</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>WCF-001-AUTHORITY-APPROVAL-PATH-REPAIR-001</t>
+          <t>P3-SYNTHESIS-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -14473,29 +14473,29 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>CERTIFIED</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>61E6AB5B881C2CE69889A7478005AAEB1AD0E6068B28A8DAACE4633B31F5143A</t>
+          <t>A456BAD939D4206681D2203DA4D0CE674D5510A7989E9EF8730820E08F76F30E</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-001-AUTHORITY-APPROVAL-PATH-REPAIR-001\bootstrap-20260919T144746651\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-SYNTHESIS-001B-IMPLEMENTATION-001\bootstrap-20260917T230506107\official-report.json</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>WCF-001-CURRENT-AUTHORITY-RATIFICATION-001</t>
+          <t>WCF-001-AUTHORITY-APPROVAL-PATH-REPAIR-001</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -14510,29 +14510,29 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>47D5F83FA798B6CEB2441DDE601A792D35DBC065E94ACDD19F3F6CCD9C0584D6</t>
+          <t>61E6AB5B881C2CE69889A7478005AAEB1AD0E6068B28A8DAACE4633B31F5143A</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-001-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260919T150059213\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-001-AUTHORITY-APPROVAL-PATH-REPAIR-001\bootstrap-20260919T144746651\official-report.json</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>WCF-002-CURRENT-AUTHORITY-RATIFICATION-001</t>
+          <t>WCF-001-CURRENT-AUTHORITY-RATIFICATION-001</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -14552,98 +14552,98 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>817BD739A8B61D20CEAE3E03FADB8350E8C9C8F28BD9714B5FD9E10679F3C78C</t>
+          <t>47D5F83FA798B6CEB2441DDE601A792D35DBC065E94ACDD19F3F6CCD9C0584D6</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-002-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260922T222135247\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-001-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260919T150059213\official-report.json</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>WCF-003-CURRENT-AUTHORITY-RATIFICATION-001</t>
+          <t>WCF-002-CURRENT-AUTHORITY-RATIFICATION-001</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>NOT_APPLICABLE</t>
+          <t>PENDING_REVIEW</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>CERTIFIED</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>5BD76C88ECF58FF03CE8DB7D85D93DA97067056517BD052BE0BCB5B86D704645</t>
+          <t>817BD739A8B61D20CEAE3E03FADB8350E8C9C8F28BD9714B5FD9E10679F3C78C</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-003-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260923T095247889\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-002-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260922T222135247\official-report.json</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>WCF-004-IMPLEMENTATION-001</t>
+          <t>WCF-003-CURRENT-AUTHORITY-RATIFICATION-001</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PENDING_REVIEW</t>
+          <t>NOT_APPLICABLE</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>8734FEA171B97F34D156A9A68A26ECCD87B1EA2F43E45F41F1A96E3861DEAD2C</t>
+          <t>5BD76C88ECF58FF03CE8DB7D85D93DA97067056517BD052BE0BCB5B86D704645</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-004-IMPLEMENTATION-001\bootstrap-20260916T114837076\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-003-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260923T095247889\official-report.json</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>WCF-008-C22-CERTIFICATION-RECONCILIATION-001</t>
+          <t>WCF-004-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -14658,29 +14658,29 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>CERTIFIED</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>D97DABE6A29700173F13B7BA5EE1CD69933995B2F5BE921A7EA5C0B9392488C5</t>
+          <t>8734FEA171B97F34D156A9A68A26ECCD87B1EA2F43E45F41F1A96E3861DEAD2C</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-008-C22-CERTIFICATION-RECONCILIATION-001\bootstrap-20260918T145858777\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-004-IMPLEMENTATION-001\bootstrap-20260916T114837076\official-report.json</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>WCF-008-CLOSURE-001</t>
+          <t>WCF-008-C22-CERTIFICATION-RECONCILIATION-001</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -14700,24 +14700,24 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>38268FB91B1ACC0FE124B0EE830AB775FB5156CF8AD8DCD64D9C87E83E54DAAB</t>
+          <t>D97DABE6A29700173F13B7BA5EE1CD69933995B2F5BE921A7EA5C0B9392488C5</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-008-CLOSURE-001\bootstrap-20260918T132849560\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-008-C22-CERTIFICATION-RECONCILIATION-001\bootstrap-20260918T145858777\official-report.json</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>WORK-AUTHORIZED-STATE-001-IMPLEMENTATION-001</t>
+          <t>WCF-008-CLOSURE-001</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -14732,59 +14732,96 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>68CD16E0D5EBF73EAAA4DFB4052029C06445CB71B431A509126A7C77F019DB14</t>
+          <t>38268FB91B1ACC0FE124B0EE830AB775FB5156CF8AD8DCD64D9C87E83E54DAAB</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WORK-AUTHORIZED-STATE-001-IMPLEMENTATION-001\bootstrap-20260916T220337699\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-008-CLOSURE-001\bootstrap-20260918T132849560\official-report.json</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-09-29 15:06:30</t>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>WORK-AUTHORIZED-STATE-001-IMPLEMENTATION-001</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>READY_FOR_REVIEW</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>PENDING_REVIEW</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>CERTIFIED</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>68CD16E0D5EBF73EAAA4DFB4052029C06445CB71B431A509126A7C77F019DB14</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>.nova-data\execution\reports\PROGRAM-003\WORK-AUTHORIZED-STATE-001-IMPLEMENTATION-001\bootstrap-20260916T220337699\official-report.json</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-10-01 00:20:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>WORK-OVERVIEW-GAP-CLOSURE-001</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>READY_FOR_REVIEW</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>PENDING_REVIEW</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>READY_FOR_REVIEW</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>D1E60A89C67587DEA5B5784E7CF402C7798ABDBC809D5108149D78055BE1535F</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>.nova-data\execution\reports\PROGRAM-003\WORK-OVERVIEW-GAP-CLOSURE-001\bootstrap-20260921T230416950\official-report.json</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>2026-09-29 15:06:30</t>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-10-01 00:20:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(work): connect Confirm to real mission runtime
</commit_message>
<xml_diff>
--- a/Docs/00_GOVERNANCE/PROJECT_TRACKING/NOVA_ROADMAP_GANTT_2026-09-29.xlsx
+++ b/Docs/00_GOVERNANCE/PROJECT_TRACKING/NOVA_ROADMAP_GANTT_2026-09-29.xlsx
@@ -13489,7 +13489,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
@@ -13526,7 +13526,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
@@ -13563,7 +13563,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
@@ -13600,7 +13600,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
@@ -13637,14 +13637,14 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NOVA-SUPER-WAVE-RT12-PROVENANCE-CLOSURE-001</t>
+          <t>NOVA-R05-CONFIRM-TO-REAL-WORK-001</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -13654,34 +13654,34 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PENDING_REVIEW</t>
+          <t>ACCEPTED</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>ACCEPTED</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CC9AD198EDB08AC8AF64CF2658789F4C7553353485A6E86D6BAB0DEBBC7D16F5</t>
+          <t>F98A222A1A40EF8AFD4F775AD3719EFBB9BA85B5D891E2ED43EE13517EF11BFB</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-SUPER-WAVE-RT12-PROVENANCE-CLOSURE-001\bootstrap-20260917T160907003\official-report.json</t>
+          <t>.nova-data\execution\reports\NOVA-AS-BUILT-COMPLETION\NOVA-R05-CONFIRM-TO-REAL-WORK-001\bootstrap-20261001T092313888\official-report.json</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NOVA-WORK-CERTIFICATION-FINAL-CLOSURE-001</t>
+          <t>NOVA-SUPER-WAVE-RT12-PROVENANCE-CLOSURE-001</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -13701,24 +13701,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>B08AC39DD5A194D049E743140B5D952C91A2262D0C1C0392B79E78A39778F888</t>
+          <t>CC9AD198EDB08AC8AF64CF2658789F4C7553353485A6E86D6BAB0DEBBC7D16F5</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-CERTIFICATION-FINAL-CLOSURE-001\bootstrap-20260919T162258742\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-SUPER-WAVE-RT12-PROVENANCE-CLOSURE-001\bootstrap-20260917T160907003\official-report.json</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>NOVA-WORK-WCF008-C19-RED-TEAM-REVALIDATION-001</t>
+          <t>NOVA-WORK-CERTIFICATION-FINAL-CLOSURE-001</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -13738,24 +13738,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>F523C276F31EBDF077F882AF67E9D65B650ED26B3497667EB547A8B560D6A8EA</t>
+          <t>B08AC39DD5A194D049E743140B5D952C91A2262D0C1C0392B79E78A39778F888</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C19-RED-TEAM-REVALIDATION-001\bootstrap-20260928T141436900\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-CERTIFICATION-FINAL-CLOSURE-001\bootstrap-20260919T162258742\official-report.json</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NOVA-WORK-WCF008-C20-OFFICIAL-REPORT-SEAL-AUDIT-001</t>
+          <t>NOVA-WORK-WCF008-C19-RED-TEAM-REVALIDATION-001</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -13775,24 +13775,24 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4C7F0ED1FD77F57332E1591404779737266EB71921180CC56BD04FF82CBB961E</t>
+          <t>F523C276F31EBDF077F882AF67E9D65B650ED26B3497667EB547A8B560D6A8EA</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C20-OFFICIAL-REPORT-SEAL-AUDIT-001\bootstrap-20260928T160351555\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C19-RED-TEAM-REVALIDATION-001\bootstrap-20260928T141436900\official-report.json</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NOVA-WORK-WCF008-C21-FINAL-CLOSURE-READINESS-001</t>
+          <t>NOVA-WORK-WCF008-C20-OFFICIAL-REPORT-SEAL-AUDIT-001</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -13807,29 +13807,29 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>22C04477C91C196702DDD99184A975A46DACDE8EBE20F6C679B1477A33861EA9</t>
+          <t>4C7F0ED1FD77F57332E1591404779737266EB71921180CC56BD04FF82CBB961E</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C21-FINAL-CLOSURE-READINESS-001\bootstrap-20260928T233841880\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C20-OFFICIAL-REPORT-SEAL-AUDIT-001\bootstrap-20260928T160351555\official-report.json</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>NOVA-WORK-WCF008-FINAL-PRE-C21-VALIDATION-001</t>
+          <t>NOVA-WORK-WCF008-C21-FINAL-CLOSURE-READINESS-001</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -13844,29 +13844,29 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>CERTIFIED</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>E23ED2A88B1C3B2650B66694C6AD9F498A1086E05DF287727C1C1EF3F74C0186</t>
+          <t>22C04477C91C196702DDD99184A975A46DACDE8EBE20F6C679B1477A33861EA9</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\NOVA\NOVA-WORK-WCF008-FINAL-PRE-C21-VALIDATION-001\bootstrap-20260928T102331010\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C21-FINAL-CLOSURE-READINESS-001\bootstrap-20260928T233841880\official-report.json</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001A-IMPLEMENTATION-CONTRACT</t>
+          <t>NOVA-WORK-WCF008-FINAL-PRE-C21-VALIDATION-001</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -13886,24 +13886,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BF26635526F1076CEAA9025E859DF3AEDFC5484E116FF1DC01B041508921B96F</t>
+          <t>E23ED2A88B1C3B2650B66694C6AD9F498A1086E05DF287727C1C1EF3F74C0186</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001A-IMPLEMENTATION-CONTRACT\bootstrap-20260908T102551406\official-report.json</t>
+          <t>.nova-data\execution\reports\NOVA\NOVA-WORK-WCF008-FINAL-PRE-C21-VALIDATION-001\bootstrap-20260928T102331010\official-report.json</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001B-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001A-IMPLEMENTATION-CONTRACT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -13918,29 +13918,29 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1D55CAFE5144E3B7EC41C6F41E7E7233A692F14EA0C15B23E5ABC7DC6D0F5CD5</t>
+          <t>BF26635526F1076CEAA9025E859DF3AEDFC5484E116FF1DC01B041508921B96F</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001B-IMPLEMENTATION-001\bootstrap-20260908T164222685\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001A-IMPLEMENTATION-CONTRACT\bootstrap-20260908T102551406\official-report.json</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001C-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -13960,24 +13960,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>351FC47C1FD4CA8E66AF7DD143A084DD1C14EB89384F00B37FFFDFD63949F352</t>
+          <t>1D55CAFE5144E3B7EC41C6F41E7E7233A692F14EA0C15B23E5ABC7DC6D0F5CD5</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001C-IMPLEMENTATION-001\bootstrap-20260910T105924679\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001B-IMPLEMENTATION-001\bootstrap-20260908T164222685\official-report.json</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001D-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001C-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -13997,24 +13997,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>27DAF65D046D7132AB457F8768ABCB22812E4ABA85BB9248B3BC79AD18C7FE29</t>
+          <t>351FC47C1FD4CA8E66AF7DD143A084DD1C14EB89384F00B37FFFDFD63949F352</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001D-IMPLEMENTATION-001\bootstrap-20260910T132750068\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001C-IMPLEMENTATION-001\bootstrap-20260910T105924679\official-report.json</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001E-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001D-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -14034,24 +14034,24 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>8B1BC8B78FAD692F07C02EEBFE3702E2BBB75CAD46E49CAD91860263389789EA</t>
+          <t>27DAF65D046D7132AB457F8768ABCB22812E4ABA85BB9248B3BC79AD18C7FE29</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001E-IMPLEMENTATION-001\bootstrap-20260910T163042722\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001D-IMPLEMENTATION-001\bootstrap-20260910T132750068\official-report.json</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001F-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001E-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -14071,24 +14071,24 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>D7B20722E39CF6C3187472CB67E23388D00419EB08E7DDD6F7C167734F515FC9</t>
+          <t>8B1BC8B78FAD692F07C02EEBFE3702E2BBB75CAD46E49CAD91860263389789EA</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001F-IMPLEMENTATION-001\bootstrap-20260910T234329189\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001E-IMPLEMENTATION-001\bootstrap-20260910T163042722\official-report.json</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001G-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001F-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -14108,24 +14108,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>5525B5851E6F2C1A8D02ADB45FAE10A6D85435164EEE5C44552E06C055395D31</t>
+          <t>D7B20722E39CF6C3187472CB67E23388D00419EB08E7DDD6F7C167734F515FC9</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001G-IMPLEMENTATION-001\bootstrap-20260913T195219085\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001F-IMPLEMENTATION-001\bootstrap-20260910T234329189\official-report.json</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>P3-BUSINESS-CERTIFICATION-001B-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001G-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -14145,24 +14145,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>32DD5DC8698BEA0E159E4C7F5E22852791A59CF119BA967C5B912823DAFF2343</t>
+          <t>5525B5851E6F2C1A8D02ADB45FAE10A6D85435164EEE5C44552E06C055395D31</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-BUSINESS-CERTIFICATION-001B-IMPLEMENTATION-001\bootstrap-20260917T150647587\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001G-IMPLEMENTATION-001\bootstrap-20260913T195219085\official-report.json</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>P3-CONFIDENCE-001B-IMPLEMENTATION-001</t>
+          <t>P3-BUSINESS-CERTIFICATION-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -14182,24 +14182,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>DB4A6A3AFAEC0C7C91C3A4E4B523603D6752A8734826F01076C249B1337706FE</t>
+          <t>32DD5DC8698BEA0E159E4C7F5E22852791A59CF119BA967C5B912823DAFF2343</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-CONFIDENCE-001B-IMPLEMENTATION-001\bootstrap-20260918T125752601\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-BUSINESS-CERTIFICATION-001B-IMPLEMENTATION-001\bootstrap-20260917T150647587\official-report.json</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>P3-EVIDENCE-001B-IMPLEMENTATION-001</t>
+          <t>P3-CONFIDENCE-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -14219,24 +14219,24 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>37A4453AA09E7157A2D12D5DF1FE0526163A252E4745435A1A18E80F9DEB29E0</t>
+          <t>DB4A6A3AFAEC0C7C91C3A4E4B523603D6752A8734826F01076C249B1337706FE</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-EVIDENCE-001B-IMPLEMENTATION-001\bootstrap-20260915T130433792\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-CONFIDENCE-001B-IMPLEMENTATION-001\bootstrap-20260918T125752601\official-report.json</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>P3-INTELLIGENCE-001B-IMPLEMENTATION-001</t>
+          <t>P3-EVIDENCE-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -14256,24 +14256,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>576375263E1D11F4D9BC49929BA0A701C645C387430AE1EAB711A1D9C71713C5</t>
+          <t>37A4453AA09E7157A2D12D5DF1FE0526163A252E4745435A1A18E80F9DEB29E0</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-INTELLIGENCE-001B-IMPLEMENTATION-001\bootstrap-20260917T205856790\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-EVIDENCE-001B-IMPLEMENTATION-001\bootstrap-20260915T130433792\official-report.json</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001C-FINAL-EVIDENCE-002</t>
+          <t>P3-INTELLIGENCE-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -14293,24 +14293,24 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>14D7FCEF0C6EE5ABAE5B3052A19508CDCD01B420EDA2E21F07120E79006B3167</t>
+          <t>576375263E1D11F4D9BC49929BA0A701C645C387430AE1EAB711A1D9C71713C5</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001C-FINAL-EVIDENCE-002\bootstrap-20260905T180227989\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-INTELLIGENCE-001B-IMPLEMENTATION-001\bootstrap-20260917T205856790\official-report.json</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001D-IMPLEMENTATION-001</t>
+          <t>P3-PLANNING-001C-FINAL-EVIDENCE-002</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -14330,24 +14330,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0442A6023581D62C7B7FA926BE258027452B03149D42C3B2AE4BA7ABBA64E243</t>
+          <t>14D7FCEF0C6EE5ABAE5B3052A19508CDCD01B420EDA2E21F07120E79006B3167</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001D-IMPLEMENTATION-001\bootstrap-20260905T190028578\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001C-FINAL-EVIDENCE-002\bootstrap-20260905T180227989\official-report.json</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001E-IMPLEMENTATION-001</t>
+          <t>P3-PLANNING-001D-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -14367,24 +14367,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>67BCE4021666AA8C5B5A2DED6BC88FD54DEF839EDA9F4ED8E28EBE76AD40D119</t>
+          <t>0442A6023581D62C7B7FA926BE258027452B03149D42C3B2AE4BA7ABBA64E243</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001E-IMPLEMENTATION-001\bootstrap-20260906T193230204\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001D-IMPLEMENTATION-001\bootstrap-20260905T190028578\official-report.json</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001F-IMPLEMENTATION-001</t>
+          <t>P3-PLANNING-001E-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -14404,24 +14404,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2D9CAF4114AE784DD95CD5471132144ADC8FADF6CACC56A94833DDF5192DE82C</t>
+          <t>67BCE4021666AA8C5B5A2DED6BC88FD54DEF839EDA9F4ED8E28EBE76AD40D119</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001F-IMPLEMENTATION-001\bootstrap-20260906T213644505\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001E-IMPLEMENTATION-001\bootstrap-20260906T193230204\official-report.json</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001G-IMPLEMENTATION-001</t>
+          <t>P3-PLANNING-001F-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -14441,24 +14441,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>B1068CA311366D7BB4DD626606C435E73F720494212448686615A821311D6DBF</t>
+          <t>2D9CAF4114AE784DD95CD5471132144ADC8FADF6CACC56A94833DDF5192DE82C</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001G-IMPLEMENTATION-001\bootstrap-20260907T174646937\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001F-IMPLEMENTATION-001\bootstrap-20260906T213644505\official-report.json</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>P3-SYNTHESIS-001B-IMPLEMENTATION-001</t>
+          <t>P3-PLANNING-001G-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -14478,24 +14478,24 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>A456BAD939D4206681D2203DA4D0CE674D5510A7989E9EF8730820E08F76F30E</t>
+          <t>B1068CA311366D7BB4DD626606C435E73F720494212448686615A821311D6DBF</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-SYNTHESIS-001B-IMPLEMENTATION-001\bootstrap-20260917T230506107\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001G-IMPLEMENTATION-001\bootstrap-20260907T174646937\official-report.json</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>WCF-001-AUTHORITY-APPROVAL-PATH-REPAIR-001</t>
+          <t>P3-SYNTHESIS-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -14510,29 +14510,29 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>CERTIFIED</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>61E6AB5B881C2CE69889A7478005AAEB1AD0E6068B28A8DAACE4633B31F5143A</t>
+          <t>A456BAD939D4206681D2203DA4D0CE674D5510A7989E9EF8730820E08F76F30E</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-001-AUTHORITY-APPROVAL-PATH-REPAIR-001\bootstrap-20260919T144746651\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-SYNTHESIS-001B-IMPLEMENTATION-001\bootstrap-20260917T230506107\official-report.json</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>WCF-001-CURRENT-AUTHORITY-RATIFICATION-001</t>
+          <t>WCF-001-AUTHORITY-APPROVAL-PATH-REPAIR-001</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -14547,29 +14547,29 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>47D5F83FA798B6CEB2441DDE601A792D35DBC065E94ACDD19F3F6CCD9C0584D6</t>
+          <t>61E6AB5B881C2CE69889A7478005AAEB1AD0E6068B28A8DAACE4633B31F5143A</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-001-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260919T150059213\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-001-AUTHORITY-APPROVAL-PATH-REPAIR-001\bootstrap-20260919T144746651\official-report.json</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>WCF-002-CURRENT-AUTHORITY-RATIFICATION-001</t>
+          <t>WCF-001-CURRENT-AUTHORITY-RATIFICATION-001</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -14589,98 +14589,98 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>817BD739A8B61D20CEAE3E03FADB8350E8C9C8F28BD9714B5FD9E10679F3C78C</t>
+          <t>47D5F83FA798B6CEB2441DDE601A792D35DBC065E94ACDD19F3F6CCD9C0584D6</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-002-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260922T222135247\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-001-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260919T150059213\official-report.json</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>WCF-003-CURRENT-AUTHORITY-RATIFICATION-001</t>
+          <t>WCF-002-CURRENT-AUTHORITY-RATIFICATION-001</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>NOT_APPLICABLE</t>
+          <t>PENDING_REVIEW</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>CERTIFIED</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>5BD76C88ECF58FF03CE8DB7D85D93DA97067056517BD052BE0BCB5B86D704645</t>
+          <t>817BD739A8B61D20CEAE3E03FADB8350E8C9C8F28BD9714B5FD9E10679F3C78C</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-003-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260923T095247889\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-002-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260922T222135247\official-report.json</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>WCF-004-IMPLEMENTATION-001</t>
+          <t>WCF-003-CURRENT-AUTHORITY-RATIFICATION-001</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PENDING_REVIEW</t>
+          <t>NOT_APPLICABLE</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>8734FEA171B97F34D156A9A68A26ECCD87B1EA2F43E45F41F1A96E3861DEAD2C</t>
+          <t>5BD76C88ECF58FF03CE8DB7D85D93DA97067056517BD052BE0BCB5B86D704645</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-004-IMPLEMENTATION-001\bootstrap-20260916T114837076\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-003-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260923T095247889\official-report.json</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>WCF-008-C22-CERTIFICATION-RECONCILIATION-001</t>
+          <t>WCF-004-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -14695,29 +14695,29 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>CERTIFIED</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>D97DABE6A29700173F13B7BA5EE1CD69933995B2F5BE921A7EA5C0B9392488C5</t>
+          <t>8734FEA171B97F34D156A9A68A26ECCD87B1EA2F43E45F41F1A96E3861DEAD2C</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-008-C22-CERTIFICATION-RECONCILIATION-001\bootstrap-20260918T145858777\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-004-IMPLEMENTATION-001\bootstrap-20260916T114837076\official-report.json</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>WCF-008-CLOSURE-001</t>
+          <t>WCF-008-C22-CERTIFICATION-RECONCILIATION-001</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -14737,24 +14737,24 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>38268FB91B1ACC0FE124B0EE830AB775FB5156CF8AD8DCD64D9C87E83E54DAAB</t>
+          <t>D97DABE6A29700173F13B7BA5EE1CD69933995B2F5BE921A7EA5C0B9392488C5</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-008-CLOSURE-001\bootstrap-20260918T132849560\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-008-C22-CERTIFICATION-RECONCILIATION-001\bootstrap-20260918T145858777\official-report.json</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>WORK-AUTHORIZED-STATE-001-IMPLEMENTATION-001</t>
+          <t>WCF-008-CLOSURE-001</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -14769,59 +14769,96 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>68CD16E0D5EBF73EAAA4DFB4052029C06445CB71B431A509126A7C77F019DB14</t>
+          <t>38268FB91B1ACC0FE124B0EE830AB775FB5156CF8AD8DCD64D9C87E83E54DAAB</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WORK-AUTHORIZED-STATE-001-IMPLEMENTATION-001\bootstrap-20260916T220337699\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-008-CLOSURE-001\bootstrap-20260918T132849560\official-report.json</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-10-01 00:20:43</t>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>WORK-AUTHORIZED-STATE-001-IMPLEMENTATION-001</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>READY_FOR_REVIEW</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>PENDING_REVIEW</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>CERTIFIED</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>68CD16E0D5EBF73EAAA4DFB4052029C06445CB71B431A509126A7C77F019DB14</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>.nova-data\execution\reports\PROGRAM-003\WORK-AUTHORIZED-STATE-001-IMPLEMENTATION-001\bootstrap-20260916T220337699\official-report.json</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-10-01 10:18:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>WORK-OVERVIEW-GAP-CLOSURE-001</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>READY_FOR_REVIEW</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>PENDING_REVIEW</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>READY_FOR_REVIEW</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>D1E60A89C67587DEA5B5784E7CF402C7798ABDBC809D5108149D78055BE1535F</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>.nova-data\execution\reports\PROGRAM-003\WORK-OVERVIEW-GAP-CLOSURE-001\bootstrap-20260921T230416950\official-report.json</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>2026-10-01 00:20:43</t>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-10-01 10:18:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(work): close R08 Work People real data path
</commit_message>
<xml_diff>
--- a/Docs/00_GOVERNANCE/PROJECT_TRACKING/NOVA_ROADMAP_GANTT_2026-09-29.xlsx
+++ b/Docs/00_GOVERNANCE/PROJECT_TRACKING/NOVA_ROADMAP_GANTT_2026-09-29.xlsx
@@ -1251,7 +1251,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1281,10 +1281,29 @@
         <f>IF(G12="Terminé","OK",IF(M12&gt;0,"RETARD",IF(TODAY()&gt;=I12,"EN COURS / À LANCER","À VENIR")))</f>
         <v/>
       </c>
-      <c r="O12" s="15" t="n"/>
+      <c r="O12" s="15" t="inlineStr">
+        <is>
+          <t>NOVA-R08-WORK-PEOPLE-REAL-PATH-EVIDENCE-RECOVERY-001</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>READY_FOR_REVIEW</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>NON RATTACHE</t>
+          <t>CLOS PAR PREUVE OFFICIELLE</t>
         </is>
       </c>
     </row>
@@ -14522,7 +14541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -14604,7 +14623,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
@@ -14641,7 +14660,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
@@ -14678,7 +14697,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
@@ -14715,7 +14734,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
@@ -14752,7 +14771,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14808,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
@@ -14826,7 +14845,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
@@ -14863,7 +14882,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
@@ -14900,51 +14919,51 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NOVA-SUPER-WAVE-RT12-PROVENANCE-CLOSURE-001</t>
+          <t>NOVA-R08-WORK-PEOPLE-REAL-PATH-001</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PENDING_REVIEW</t>
+          <t>REJECTED</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>REJECTED</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CC9AD198EDB08AC8AF64CF2658789F4C7553353485A6E86D6BAB0DEBBC7D16F5</t>
+          <t>0C7038A014071A526F3C4C9B63EAC6125D77C1A6A0DCFD7D98BFB27397BCC7BD</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-SUPER-WAVE-RT12-PROVENANCE-CLOSURE-001\bootstrap-20260917T160907003\official-report.json</t>
+          <t>tools\cerebrau\reports\missions\NOVA-R08-WORK-PEOPLE-REAL-PATH-001\bootstrap-20261003T180129549\official-report.json</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>NOVA-WORK-CERTIFICATION-FINAL-CLOSURE-001</t>
+          <t>NOVA-R08-WORK-PEOPLE-REAL-PATH-EVIDENCE-RECOVERY-001</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -14954,34 +14973,34 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>PENDING_REVIEW</t>
+          <t>ACCEPTED</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>ACCEPTED</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>B08AC39DD5A194D049E743140B5D952C91A2262D0C1C0392B79E78A39778F888</t>
+          <t>D2A060F8AC39D1E000FB48D39CFC740401FEB566AC2AD625D94373CEDA999D8F</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-CERTIFICATION-FINAL-CLOSURE-001\bootstrap-20260919T162258742\official-report.json</t>
+          <t>tools\cerebrau\reports\missions\NOVA-R08-WORK-PEOPLE-REAL-PATH-EVIDENCE-RECOVERY-001\bootstrap-20261004T113052217\official-report.json</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NOVA-WORK-WCF008-C19-RED-TEAM-REVALIDATION-001</t>
+          <t>NOVA-SUPER-WAVE-RT12-PROVENANCE-CLOSURE-001</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -15001,24 +15020,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>F523C276F31EBDF077F882AF67E9D65B650ED26B3497667EB547A8B560D6A8EA</t>
+          <t>CC9AD198EDB08AC8AF64CF2658789F4C7553353485A6E86D6BAB0DEBBC7D16F5</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C19-RED-TEAM-REVALIDATION-001\bootstrap-20260928T141436900\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-SUPER-WAVE-RT12-PROVENANCE-CLOSURE-001\bootstrap-20260917T160907003\official-report.json</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NOVA-WORK-WCF008-C20-OFFICIAL-REPORT-SEAL-AUDIT-001</t>
+          <t>NOVA-WORK-CERTIFICATION-FINAL-CLOSURE-001</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -15038,24 +15057,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>4C7F0ED1FD77F57332E1591404779737266EB71921180CC56BD04FF82CBB961E</t>
+          <t>B08AC39DD5A194D049E743140B5D952C91A2262D0C1C0392B79E78A39778F888</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C20-OFFICIAL-REPORT-SEAL-AUDIT-001\bootstrap-20260928T160351555\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-CERTIFICATION-FINAL-CLOSURE-001\bootstrap-20260919T162258742\official-report.json</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NOVA-WORK-WCF008-C21-FINAL-CLOSURE-READINESS-001</t>
+          <t>NOVA-WORK-WCF008-C19-RED-TEAM-REVALIDATION-001</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -15070,29 +15089,29 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>22C04477C91C196702DDD99184A975A46DACDE8EBE20F6C679B1477A33861EA9</t>
+          <t>F523C276F31EBDF077F882AF67E9D65B650ED26B3497667EB547A8B560D6A8EA</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C21-FINAL-CLOSURE-READINESS-001\bootstrap-20260928T233841880\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C19-RED-TEAM-REVALIDATION-001\bootstrap-20260928T141436900\official-report.json</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>NOVA-WORK-WCF008-FINAL-PRE-C21-VALIDATION-001</t>
+          <t>NOVA-WORK-WCF008-C20-OFFICIAL-REPORT-SEAL-AUDIT-001</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -15112,24 +15131,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>E23ED2A88B1C3B2650B66694C6AD9F498A1086E05DF287727C1C1EF3F74C0186</t>
+          <t>4C7F0ED1FD77F57332E1591404779737266EB71921180CC56BD04FF82CBB961E</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\NOVA\NOVA-WORK-WCF008-FINAL-PRE-C21-VALIDATION-001\bootstrap-20260928T102331010\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C20-OFFICIAL-REPORT-SEAL-AUDIT-001\bootstrap-20260928T160351555\official-report.json</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001A-IMPLEMENTATION-CONTRACT</t>
+          <t>NOVA-WORK-WCF008-C21-FINAL-CLOSURE-READINESS-001</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -15144,29 +15163,29 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>CERTIFIED</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BF26635526F1076CEAA9025E859DF3AEDFC5484E116FF1DC01B041508921B96F</t>
+          <t>22C04477C91C196702DDD99184A975A46DACDE8EBE20F6C679B1477A33861EA9</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001A-IMPLEMENTATION-CONTRACT\bootstrap-20260908T102551406\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\NOVA-WORK-WCF008-C21-FINAL-CLOSURE-READINESS-001\bootstrap-20260928T233841880\official-report.json</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001B-IMPLEMENTATION-001</t>
+          <t>NOVA-WORK-WCF008-FINAL-PRE-C21-VALIDATION-001</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -15181,29 +15200,29 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1D55CAFE5144E3B7EC41C6F41E7E7233A692F14EA0C15B23E5ABC7DC6D0F5CD5</t>
+          <t>E23ED2A88B1C3B2650B66694C6AD9F498A1086E05DF287727C1C1EF3F74C0186</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001B-IMPLEMENTATION-001\bootstrap-20260908T164222685\official-report.json</t>
+          <t>.nova-data\execution\reports\NOVA\NOVA-WORK-WCF008-FINAL-PRE-C21-VALIDATION-001\bootstrap-20260928T102331010\official-report.json</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001C-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001A-IMPLEMENTATION-CONTRACT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -15218,29 +15237,29 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>351FC47C1FD4CA8E66AF7DD143A084DD1C14EB89384F00B37FFFDFD63949F352</t>
+          <t>BF26635526F1076CEAA9025E859DF3AEDFC5484E116FF1DC01B041508921B96F</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001C-IMPLEMENTATION-001\bootstrap-20260910T105924679\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001A-IMPLEMENTATION-CONTRACT\bootstrap-20260908T102551406\official-report.json</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001D-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -15260,24 +15279,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>27DAF65D046D7132AB457F8768ABCB22812E4ABA85BB9248B3BC79AD18C7FE29</t>
+          <t>1D55CAFE5144E3B7EC41C6F41E7E7233A692F14EA0C15B23E5ABC7DC6D0F5CD5</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001D-IMPLEMENTATION-001\bootstrap-20260910T132750068\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001B-IMPLEMENTATION-001\bootstrap-20260908T164222685\official-report.json</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001E-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001C-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -15297,24 +15316,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>8B1BC8B78FAD692F07C02EEBFE3702E2BBB75CAD46E49CAD91860263389789EA</t>
+          <t>351FC47C1FD4CA8E66AF7DD143A084DD1C14EB89384F00B37FFFDFD63949F352</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001E-IMPLEMENTATION-001\bootstrap-20260910T163042722\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001C-IMPLEMENTATION-001\bootstrap-20260910T105924679\official-report.json</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001F-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001D-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -15334,24 +15353,24 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>D7B20722E39CF6C3187472CB67E23388D00419EB08E7DDD6F7C167734F515FC9</t>
+          <t>27DAF65D046D7132AB457F8768ABCB22812E4ABA85BB9248B3BC79AD18C7FE29</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001F-IMPLEMENTATION-001\bootstrap-20260910T234329189\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001D-IMPLEMENTATION-001\bootstrap-20260910T132750068\official-report.json</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>P3-ACTIONS-001G-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001E-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -15371,24 +15390,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>5525B5851E6F2C1A8D02ADB45FAE10A6D85435164EEE5C44552E06C055395D31</t>
+          <t>8B1BC8B78FAD692F07C02EEBFE3702E2BBB75CAD46E49CAD91860263389789EA</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001G-IMPLEMENTATION-001\bootstrap-20260913T195219085\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001E-IMPLEMENTATION-001\bootstrap-20260910T163042722\official-report.json</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>P3-BUSINESS-CERTIFICATION-001B-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001F-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -15408,24 +15427,24 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>32DD5DC8698BEA0E159E4C7F5E22852791A59CF119BA967C5B912823DAFF2343</t>
+          <t>D7B20722E39CF6C3187472CB67E23388D00419EB08E7DDD6F7C167734F515FC9</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-BUSINESS-CERTIFICATION-001B-IMPLEMENTATION-001\bootstrap-20260917T150647587\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001F-IMPLEMENTATION-001\bootstrap-20260910T234329189\official-report.json</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P3-CONFIDENCE-001B-IMPLEMENTATION-001</t>
+          <t>P3-ACTIONS-001G-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -15445,24 +15464,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>DB4A6A3AFAEC0C7C91C3A4E4B523603D6752A8734826F01076C249B1337706FE</t>
+          <t>5525B5851E6F2C1A8D02ADB45FAE10A6D85435164EEE5C44552E06C055395D31</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-CONFIDENCE-001B-IMPLEMENTATION-001\bootstrap-20260918T125752601\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-ACTIONS-001G-IMPLEMENTATION-001\bootstrap-20260913T195219085\official-report.json</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>P3-EVIDENCE-001B-IMPLEMENTATION-001</t>
+          <t>P3-BUSINESS-CERTIFICATION-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -15482,24 +15501,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>37A4453AA09E7157A2D12D5DF1FE0526163A252E4745435A1A18E80F9DEB29E0</t>
+          <t>32DD5DC8698BEA0E159E4C7F5E22852791A59CF119BA967C5B912823DAFF2343</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-EVIDENCE-001B-IMPLEMENTATION-001\bootstrap-20260915T130433792\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-BUSINESS-CERTIFICATION-001B-IMPLEMENTATION-001\bootstrap-20260917T150647587\official-report.json</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>P3-INTELLIGENCE-001B-IMPLEMENTATION-001</t>
+          <t>P3-CONFIDENCE-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -15519,24 +15538,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>576375263E1D11F4D9BC49929BA0A701C645C387430AE1EAB711A1D9C71713C5</t>
+          <t>DB4A6A3AFAEC0C7C91C3A4E4B523603D6752A8734826F01076C249B1337706FE</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-INTELLIGENCE-001B-IMPLEMENTATION-001\bootstrap-20260917T205856790\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-CONFIDENCE-001B-IMPLEMENTATION-001\bootstrap-20260918T125752601\official-report.json</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001C-FINAL-EVIDENCE-002</t>
+          <t>P3-EVIDENCE-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -15556,24 +15575,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>14D7FCEF0C6EE5ABAE5B3052A19508CDCD01B420EDA2E21F07120E79006B3167</t>
+          <t>37A4453AA09E7157A2D12D5DF1FE0526163A252E4745435A1A18E80F9DEB29E0</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001C-FINAL-EVIDENCE-002\bootstrap-20260905T180227989\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-EVIDENCE-001B-IMPLEMENTATION-001\bootstrap-20260915T130433792\official-report.json</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001D-IMPLEMENTATION-001</t>
+          <t>P3-INTELLIGENCE-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -15593,24 +15612,24 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>0442A6023581D62C7B7FA926BE258027452B03149D42C3B2AE4BA7ABBA64E243</t>
+          <t>576375263E1D11F4D9BC49929BA0A701C645C387430AE1EAB711A1D9C71713C5</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001D-IMPLEMENTATION-001\bootstrap-20260905T190028578\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-INTELLIGENCE-001B-IMPLEMENTATION-001\bootstrap-20260917T205856790\official-report.json</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001E-IMPLEMENTATION-001</t>
+          <t>P3-PLANNING-001C-FINAL-EVIDENCE-002</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -15630,24 +15649,24 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>67BCE4021666AA8C5B5A2DED6BC88FD54DEF839EDA9F4ED8E28EBE76AD40D119</t>
+          <t>14D7FCEF0C6EE5ABAE5B3052A19508CDCD01B420EDA2E21F07120E79006B3167</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001E-IMPLEMENTATION-001\bootstrap-20260906T193230204\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001C-FINAL-EVIDENCE-002\bootstrap-20260905T180227989\official-report.json</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001F-IMPLEMENTATION-001</t>
+          <t>P3-PLANNING-001D-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -15667,24 +15686,24 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2D9CAF4114AE784DD95CD5471132144ADC8FADF6CACC56A94833DDF5192DE82C</t>
+          <t>0442A6023581D62C7B7FA926BE258027452B03149D42C3B2AE4BA7ABBA64E243</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001F-IMPLEMENTATION-001\bootstrap-20260906T213644505\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001D-IMPLEMENTATION-001\bootstrap-20260905T190028578\official-report.json</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>P3-PLANNING-001G-IMPLEMENTATION-001</t>
+          <t>P3-PLANNING-001E-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -15704,24 +15723,24 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>B1068CA311366D7BB4DD626606C435E73F720494212448686615A821311D6DBF</t>
+          <t>67BCE4021666AA8C5B5A2DED6BC88FD54DEF839EDA9F4ED8E28EBE76AD40D119</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001G-IMPLEMENTATION-001\bootstrap-20260907T174646937\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001E-IMPLEMENTATION-001\bootstrap-20260906T193230204\official-report.json</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>P3-SYNTHESIS-001B-IMPLEMENTATION-001</t>
+          <t>P3-PLANNING-001F-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -15741,24 +15760,24 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>A456BAD939D4206681D2203DA4D0CE674D5510A7989E9EF8730820E08F76F30E</t>
+          <t>2D9CAF4114AE784DD95CD5471132144ADC8FADF6CACC56A94833DDF5192DE82C</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\P3-SYNTHESIS-001B-IMPLEMENTATION-001\bootstrap-20260917T230506107\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001F-IMPLEMENTATION-001\bootstrap-20260906T213644505\official-report.json</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>WCF-001-AUTHORITY-APPROVAL-PATH-REPAIR-001</t>
+          <t>P3-PLANNING-001G-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -15773,29 +15792,29 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>CERTIFIED</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>61E6AB5B881C2CE69889A7478005AAEB1AD0E6068B28A8DAACE4633B31F5143A</t>
+          <t>B1068CA311366D7BB4DD626606C435E73F720494212448686615A821311D6DBF</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-001-AUTHORITY-APPROVAL-PATH-REPAIR-001\bootstrap-20260919T144746651\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-PLANNING-001G-IMPLEMENTATION-001\bootstrap-20260907T174646937\official-report.json</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>WCF-001-CURRENT-AUTHORITY-RATIFICATION-001</t>
+          <t>P3-SYNTHESIS-001B-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -15815,24 +15834,24 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>47D5F83FA798B6CEB2441DDE601A792D35DBC065E94ACDD19F3F6CCD9C0584D6</t>
+          <t>A456BAD939D4206681D2203DA4D0CE674D5510A7989E9EF8730820E08F76F30E</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-001-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260919T150059213\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\P3-SYNTHESIS-001B-IMPLEMENTATION-001\bootstrap-20260917T230506107\official-report.json</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>WCF-002-CURRENT-AUTHORITY-RATIFICATION-001</t>
+          <t>WCF-001-AUTHORITY-APPROVAL-PATH-REPAIR-001</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -15847,66 +15866,66 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>817BD739A8B61D20CEAE3E03FADB8350E8C9C8F28BD9714B5FD9E10679F3C78C</t>
+          <t>61E6AB5B881C2CE69889A7478005AAEB1AD0E6068B28A8DAACE4633B31F5143A</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-002-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260922T222135247\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-001-AUTHORITY-APPROVAL-PATH-REPAIR-001\bootstrap-20260919T144746651\official-report.json</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>WCF-003-CURRENT-AUTHORITY-RATIFICATION-001</t>
+          <t>WCF-001-CURRENT-AUTHORITY-RATIFICATION-001</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>NOT_APPLICABLE</t>
+          <t>PENDING_REVIEW</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>CERTIFIED</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>5BD76C88ECF58FF03CE8DB7D85D93DA97067056517BD052BE0BCB5B86D704645</t>
+          <t>47D5F83FA798B6CEB2441DDE601A792D35DBC065E94ACDD19F3F6CCD9C0584D6</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-003-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260923T095247889\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-001-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260919T150059213\official-report.json</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>WCF-004-IMPLEMENTATION-001</t>
+          <t>WCF-002-CURRENT-AUTHORITY-RATIFICATION-001</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -15926,61 +15945,61 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>8734FEA171B97F34D156A9A68A26ECCD87B1EA2F43E45F41F1A96E3861DEAD2C</t>
+          <t>817BD739A8B61D20CEAE3E03FADB8350E8C9C8F28BD9714B5FD9E10679F3C78C</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-004-IMPLEMENTATION-001\bootstrap-20260916T114837076\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-002-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260922T222135247\official-report.json</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>WCF-008-C22-CERTIFICATION-RECONCILIATION-001</t>
+          <t>WCF-003-CURRENT-AUTHORITY-RATIFICATION-001</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PENDING_REVIEW</t>
+          <t>NOT_APPLICABLE</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>D97DABE6A29700173F13B7BA5EE1CD69933995B2F5BE921A7EA5C0B9392488C5</t>
+          <t>5BD76C88ECF58FF03CE8DB7D85D93DA97067056517BD052BE0BCB5B86D704645</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-008-C22-CERTIFICATION-RECONCILIATION-001\bootstrap-20260918T145858777\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-003-CURRENT-AUTHORITY-RATIFICATION-001\bootstrap-20260923T095247889\official-report.json</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>WCF-008-CLOSURE-001</t>
+          <t>WCF-004-IMPLEMENTATION-001</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -15995,29 +16014,29 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>READY_FOR_REVIEW</t>
+          <t>CERTIFIED</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>38268FB91B1ACC0FE124B0EE830AB775FB5156CF8AD8DCD64D9C87E83E54DAAB</t>
+          <t>8734FEA171B97F34D156A9A68A26ECCD87B1EA2F43E45F41F1A96E3861DEAD2C</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WCF-008-CLOSURE-001\bootstrap-20260918T132849560\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-004-IMPLEMENTATION-001\bootstrap-20260916T114837076\official-report.json</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>WORK-AUTHORIZED-STATE-001-IMPLEMENTATION-001</t>
+          <t>WCF-008-C22-CERTIFICATION-RECONCILIATION-001</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -16032,59 +16051,133 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>CERTIFIED</t>
+          <t>READY_FOR_REVIEW</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>68CD16E0D5EBF73EAAA4DFB4052029C06445CB71B431A509126A7C77F019DB14</t>
+          <t>D97DABE6A29700173F13B7BA5EE1CD69933995B2F5BE921A7EA5C0B9392488C5</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>.nova-data\execution\reports\PROGRAM-003\WORK-AUTHORIZED-STATE-001-IMPLEMENTATION-001\bootstrap-20260916T220337699\official-report.json</t>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-008-C22-CERTIFICATION-RECONCILIATION-001\bootstrap-20260918T145858777\official-report.json</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-10-02 23:33:41</t>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>WCF-008-CLOSURE-001</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>READY_FOR_REVIEW</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>PENDING_REVIEW</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>READY_FOR_REVIEW</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>38268FB91B1ACC0FE124B0EE830AB775FB5156CF8AD8DCD64D9C87E83E54DAAB</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>.nova-data\execution\reports\PROGRAM-003\WCF-008-CLOSURE-001\bootstrap-20260918T132849560\official-report.json</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-10-04 23:35:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>WORK-AUTHORIZED-STATE-001-IMPLEMENTATION-001</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>READY_FOR_REVIEW</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>PENDING_REVIEW</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>CERTIFIED</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>68CD16E0D5EBF73EAAA4DFB4052029C06445CB71B431A509126A7C77F019DB14</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>.nova-data\execution\reports\PROGRAM-003\WORK-AUTHORIZED-STATE-001-IMPLEMENTATION-001\bootstrap-20260916T220337699\official-report.json</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-10-04 23:35:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>WORK-OVERVIEW-GAP-CLOSURE-001</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>READY_FOR_REVIEW</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>PENDING_REVIEW</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>READY_FOR_REVIEW</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>D1E60A89C67587DEA5B5784E7CF402C7798ABDBC809D5108149D78055BE1535F</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>.nova-data\execution\reports\PROGRAM-003\WORK-OVERVIEW-GAP-CLOSURE-001\bootstrap-20260921T230416950\official-report.json</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>2026-10-02 23:33:41</t>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-10-04 23:35:10</t>
         </is>
       </c>
     </row>

</xml_diff>